<commit_message>
DIO - Aplicativo de investimentos
Projeto de aplicativo de investimentos desenvolvido com base nas diretrizes do bootcamp da DIO, com ênfase no uso de Excel e Inteligência Artificial. 

O objetivo é simular diferentes cenários de investimento em múltiplas aplicações, adotando como parâmetro o perfil do investidor.
</commit_message>
<xml_diff>
--- a/App_Investimentos.xlsx
+++ b/App_Investimentos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/217cc67307c45ea1/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="13_ncr:1_{AA77CDAA-366C-4305-9366-5619397C2ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8142D5CE-75E9-406F-8756-0A29E0C3EAE5}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="13_ncr:1_{AA77CDAA-366C-4305-9366-5619397C2ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4935ADB3-3074-4C1A-9E90-43A947758742}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="0" xr2:uid="{5D7F3A9A-47AD-4D1B-B95A-5B68640EB23A}"/>
   </bookViews>
@@ -602,10 +602,10 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="101"/>
+      <c14:style val="102"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="1"/>
+      <c:style val="2"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
@@ -635,16 +635,13 @@
               <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="88500"/>
+                    <a:schemeClr val="accent2">
                       <a:lumMod val="60000"/>
                       <a:lumOff val="40000"/>
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="88500"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="accent2"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="0"/>
@@ -669,16 +666,13 @@
               <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="55000"/>
+                    <a:schemeClr val="accent4">
                       <a:lumMod val="60000"/>
                       <a:lumOff val="40000"/>
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="55000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="accent4"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="0"/>
@@ -703,16 +697,13 @@
               <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="75000"/>
+                    <a:schemeClr val="accent6">
                       <a:lumMod val="60000"/>
                       <a:lumOff val="40000"/>
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="75000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="accent6"/>
                   </a:gs>
                 </a:gsLst>
                 <a:lin ang="5400000" scaled="0"/>
@@ -737,15 +728,15 @@
               <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="98500"/>
+                    <a:schemeClr val="accent2">
+                      <a:lumMod val="60000"/>
                       <a:lumMod val="60000"/>
                       <a:lumOff val="40000"/>
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="98500"/>
+                    <a:schemeClr val="accent2">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:gs>
                 </a:gsLst>
@@ -771,15 +762,15 @@
               <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="30000"/>
+                    <a:schemeClr val="accent4">
+                      <a:lumMod val="60000"/>
                       <a:lumMod val="60000"/>
                       <a:lumOff val="40000"/>
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="30000"/>
+                    <a:schemeClr val="accent4">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:gs>
                 </a:gsLst>
@@ -805,15 +796,15 @@
               <a:gradFill>
                 <a:gsLst>
                   <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="60000"/>
+                    <a:schemeClr val="accent6">
+                      <a:lumMod val="60000"/>
                       <a:lumMod val="60000"/>
                       <a:lumOff val="40000"/>
                     </a:schemeClr>
                   </a:gs>
                   <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:tint val="60000"/>
+                    <a:schemeClr val="accent6">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:gs>
                 </a:gsLst>
@@ -918,22 +909,22 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.3</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1</c:v>
+                  <c:v>0.05</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1</c:v>
+                  <c:v>0.05</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1030,28 +1021,38 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="20">
-  <a:schemeClr val="dk1"/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="12">
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
   <cs:variation>
-    <a:tint val="88500"/>
+    <a:lumMod val="60000"/>
   </cs:variation>
   <cs:variation>
-    <a:tint val="55000"/>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
   </cs:variation>
   <cs:variation>
-    <a:tint val="75000"/>
+    <a:lumMod val="80000"/>
   </cs:variation>
   <cs:variation>
-    <a:tint val="98500"/>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
   </cs:variation>
   <cs:variation>
-    <a:tint val="30000"/>
+    <a:lumMod val="50000"/>
   </cs:variation>
   <cs:variation>
-    <a:tint val="60000"/>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
   </cs:variation>
   <cs:variation>
-    <a:tint val="80000"/>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
   </cs:variation>
 </cs:colorStyle>
 </file>
@@ -2090,8 +2091,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9D1864F-2207-42A9-A2FD-784020E63C3E}">
-  <dimension ref="A5:E35"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="18" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="30.7109375" style="7" customWidth="1"/>
@@ -2099,6 +2100,10 @@
     <col min="6" max="16384" width="13.28515625" style="7" hidden="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25"/>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="34" t="s">
         <v>0</v>
@@ -2313,7 +2318,7 @@
       </c>
       <c r="C25" s="33"/>
       <c r="D25" s="26" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:4" s="21" customFormat="1" x14ac:dyDescent="0.25">
@@ -2327,6 +2332,7 @@
         <v>800</v>
       </c>
     </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:4" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="18"/>
       <c r="B28" s="4" t="s">
@@ -2345,11 +2351,11 @@
       </c>
       <c r="C29" s="28">
         <f>VLOOKUP($D$25&amp;"-"&amp;$B29,Auxiliar!$A:$D,4,FALSE)</f>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D29" s="16">
         <f t="shared" ref="D29:D34" si="0">C29*$D$26</f>
-        <v>240</v>
+        <v>400</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -2358,11 +2364,11 @@
       </c>
       <c r="C30" s="28">
         <f>VLOOKUP($D$25&amp;"-"&amp;$B30,Auxiliar!$A:$D,4,FALSE)</f>
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D30" s="16">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -2371,11 +2377,11 @@
       </c>
       <c r="C31" s="28">
         <f>VLOOKUP($D$25&amp;"-"&amp;$B31,Auxiliar!$A:$D,4,FALSE)</f>
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="D31" s="16">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -2384,11 +2390,11 @@
       </c>
       <c r="C32" s="28">
         <f>VLOOKUP($D$25&amp;"-"&amp;$B32,Auxiliar!$A:$D,4,FALSE)</f>
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="D32" s="16">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
@@ -2397,11 +2403,11 @@
       </c>
       <c r="C33" s="28">
         <f>VLOOKUP($D$25&amp;"-"&amp;$B33,Auxiliar!$A:$D,4,FALSE)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D33" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
@@ -2410,11 +2416,11 @@
       </c>
       <c r="C34" s="28">
         <f>VLOOKUP($D$25&amp;"-"&amp;$B34,Auxiliar!$A:$D,4,FALSE)</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D34" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
@@ -2427,6 +2433,21 @@
         <v>800</v>
       </c>
     </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25"/>
+    <row r="49" x14ac:dyDescent="0.25"/>
+    <row r="50" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B26:C26"/>

</xml_diff>